<commit_message>
Fix portfolio downloads and contact flow
</commit_message>
<xml_diff>
--- a/projects/ai-outreach-hub/AI_Outreach_Hub.xlsx
+++ b/projects/ai-outreach-hub/AI_Outreach_Hub.xlsx
@@ -2,44 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R3747495c87a44c66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="2" r:id="Rfc667b3abd714bbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="Rcf90434867f049e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="4" r:id="Rabbdabe1132e4a5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Templates" sheetId="5" r:id="R65e431af70fa4526"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R2c90a47d52ab4f14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="2" r:id="R2eee35b7691f4702"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="R54286f27d8d04299"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="4" r:id="R3013d1970a8e438d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Templates" sheetId="5" r:id="R050a311a5e2b447c"/>
   </x:sheets>
 </x:workbook>
-</file>
-
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:authors>
-    <x:author>tc={19C0D145-2020-C563-AA01-D74D24B3229D}</x:author>
-    <x:author>tc={F28E6101-3188-CA9B-1C4C-E942D45A2995}</x:author>
-  </x:authors>
-  <x:commentList>
-    <x:comment ref="G5" authorId="0">
-      <x:text>
-        <x:r>
-          <x:t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Source URL is mandatory so every claim and contact can be audited.</x:t>
-        </x:r>
-      </x:text>
-    </x:comment>
-    <x:comment ref="P5" authorId="1">
-      <x:text>
-        <x:r>
-          <x:t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Apps Script only processes DRAFT_READY rows and writes Gmail drafts; it never sends automatically.</x:t>
-        </x:r>
-      </x:text>
-    </x:comment>
-  </x:commentList>
-</x:comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -690,12 +659,6 @@
 </x:styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Kirill" id="{CD007003-3FE2-4FFE-8721-BD4F45514918}"/>
-</xltc:personList>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LeadsTable" displayName="LeadsTable" ref="A5:R205" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="18">
@@ -931,17 +894,6 @@
 </a:theme>
 </file>
 
-<file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
-<xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="G5" dT="2026-08-11T17:18:39.849" personId="{CD007003-3FE2-4FFE-8721-BD4F45514918}" id="{19C0D145-2020-C563-AA01-D74D24B3229D}">
-    <xltc:text>Source URL is mandatory so every claim and contact can be audited.</xltc:text>
-  </xltc:threadedComment>
-  <xltc:threadedComment ref="P5" dT="2026-08-11T17:18:39.85" personId="{CD007003-3FE2-4FFE-8721-BD4F45514918}" id="{F28E6101-3188-CA9B-1C4C-E942D45A2995}">
-    <xltc:text>Apps Script only processes DRAFT_READY rows and writes Gmail drafts; it never sends automatically.</xltc:text>
-  </xltc:threadedComment>
-</xltc:ThreadedComments>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -1412,7 +1364,7 @@
     <x:mergeCell ref="E5:G6"/>
     <x:mergeCell ref="I5:K6"/>
     <x:mergeCell ref="M5:N6"/>
-    <x:mergeCell ref="A9:F9"/>
+    <x:mergeCell ref="A9:B9"/>
     <x:mergeCell ref="D9:N9"/>
     <x:mergeCell ref="D10:N18"/>
     <x:mergeCell ref="A22:N22"/>
@@ -6135,9 +6087,8 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad35ff7270e84494"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36cdc72b82f14e7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R642d0edfa7d64770"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8645,7 +8596,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14c95d5643ed4b25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96cf9d61dc1d4d40"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>